<commit_message>
Add GBD permanent links
</commit_message>
<xml_diff>
--- a/data/processed/Karlsson2025_GBD_US_mapping_final.xlsx
+++ b/data/processed/Karlsson2025_GBD_US_mapping_final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/04Dissertation/uw-phd-aim1/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_2843014730D8E00CF9A01B6AF2558D30C2FE69D2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{489FE319-F541-400B-A736-1B3C56D0BB1B}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="11_2843014730D8E00CF9A01B6AF2558D30C2FE69D2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68A41CE0-294C-4F6D-8BE9-C73683C0D395}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,48 @@
     <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Condition_GBD_mapping!$A$1:$E$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Condition_GBD_mapping!$A$1:$F$34</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>WILLIAM GARCIA</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{0CE08529-516F-43E0-BED3-1DF3D62E2B01}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>WILLIAM GARCIA:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Each color higligth the block consilted in GBD. Each block is a different permanent link for replication purposes</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="142">
   <si>
     <t>Karlsson_2025_priority_condition</t>
   </si>
@@ -305,12 +339,6 @@
     <t>NCHS/CDC: Alzheimer's disease; Parkinson disease; other nervous system disorders</t>
   </si>
   <si>
-    <t>Violence</t>
-  </si>
-  <si>
-    <t>May overlap with homicide definitions</t>
-  </si>
-  <si>
     <t>Cardiovascular diseases (excluding NCD-7)</t>
   </si>
   <si>
@@ -354,13 +382,115 @@
   </si>
   <si>
     <t>Final verification completed against the Karlsson supplemental table image. All I-8 and NCD-7 categories appearing in the figure/table were checked and included.</t>
+  </si>
+  <si>
+    <t>Chronic kidney disease due to diabetes</t>
+  </si>
+  <si>
+    <t>Explicitly listed in Karlsson supplemental table under Diabetes</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Chronic kidney disease due to diabetes</t>
+  </si>
+  <si>
+    <t>NCDs strongly linked to infections</t>
+  </si>
+  <si>
+    <t>Cervical cancer</t>
+  </si>
+  <si>
+    <t>HPV-related cancer</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Cervical cancer</t>
+  </si>
+  <si>
+    <t>Cirrhosis due to hepatitis B</t>
+  </si>
+  <si>
+    <t>HBV-related cirrhosis</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Chronic liver disease and cirrhosis</t>
+  </si>
+  <si>
+    <t>Cirrhosis due to hepatitis C</t>
+  </si>
+  <si>
+    <t>HCV-related cirrhosis</t>
+  </si>
+  <si>
+    <t>Liver cancer secondary to hepatitis B</t>
+  </si>
+  <si>
+    <t>HBV-related liver cancer</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Liver and intrahepatic bile duct cancer</t>
+  </si>
+  <si>
+    <t>Liver cancer secondary to hepatitis C</t>
+  </si>
+  <si>
+    <t>HCV-related liver cancer</t>
+  </si>
+  <si>
+    <t>Rheumatic heart disease</t>
+  </si>
+  <si>
+    <t>Post-streptococcal chronic cardiovascular disease</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Rheumatic heart disease</t>
+  </si>
+  <si>
+    <t>Stomach cancer</t>
+  </si>
+  <si>
+    <t>Often H. pylori-associated</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Stomach cancer</t>
+  </si>
+  <si>
+    <t>NCDs strongly linked to tobacco use</t>
+  </si>
+  <si>
+    <t>Larynx cancer</t>
+  </si>
+  <si>
+    <t>Tobacco-related malignancy</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Malignant neoplasm of larynx</t>
+  </si>
+  <si>
+    <t>Mouth and oropharynx cancer</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Oral cavity and pharynx cancers</t>
+  </si>
+  <si>
+    <t>Trachea, bronchus, and lung cancer</t>
+  </si>
+  <si>
+    <t>Major smoking-related cancer group</t>
+  </si>
+  <si>
+    <t>NCHS/CDC: Lung cancer</t>
+  </si>
+  <si>
+    <t>Cause - Optional extension</t>
+  </si>
+  <si>
+    <t>Relevant for US state-level decomposition. May overlap with homicide definitions</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -379,8 +509,35 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -395,6 +552,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -435,7 +616,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -456,6 +637,27 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -759,8 +961,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F26"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1015,7 +1217,7 @@
       <c r="A13" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="8" t="s">
         <v>40</v>
       </c>
       <c r="C13" s="3" t="s">
@@ -1035,7 +1237,7 @@
       <c r="A14" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="8" t="s">
         <v>44</v>
       </c>
       <c r="C14" s="3" t="s">
@@ -1055,7 +1257,7 @@
       <c r="A15" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="8" t="s">
         <v>49</v>
       </c>
       <c r="C15" s="3" t="s">
@@ -1071,38 +1273,38 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>54</v>
+        <v>48</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>108</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>55</v>
+        <v>109</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>56</v>
+        <v>110</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>58</v>
+      <c r="B17" s="8" t="s">
+        <v>54</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>56</v>
@@ -1111,32 +1313,32 @@
         <v>57</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>61</v>
+    <row r="18" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>66</v>
+        <v>60</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>61</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>8</v>
@@ -1145,38 +1347,38 @@
         <v>62</v>
       </c>
       <c r="E19" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
+    <row r="21" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B21" s="11" t="s">
         <v>70</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>71</v>
@@ -1185,37 +1387,37 @@
         <v>72</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F21" s="5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A22" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>82</v>
+    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="12" t="s">
         <v>85</v>
       </c>
       <c r="C23" s="5" t="s">
@@ -1232,10 +1434,10 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="12" t="s">
         <v>90</v>
       </c>
       <c r="C24" s="5" t="s">
@@ -1253,47 +1455,249 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B32" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>135</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="5" t="s">
+      <c r="B35" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="E25" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
+      <c r="C35" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="E35" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="F35" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="E26" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>100</v>
+    </row>
+    <row r="36" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A36" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D36" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E36" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F36" s="5" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F34" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1307,47 +1711,47 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add references and causes groupings
</commit_message>
<xml_diff>
--- a/data/processed/Karlsson2025_GBD_US_mapping_final.xlsx
+++ b/data/processed/Karlsson2025_GBD_US_mapping_final.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/04Dissertation/uw-phd-aim1/data/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="11_2843014730D8E00CF9A01B6AF2558D30C2FE69D2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{68A41CE0-294C-4F6D-8BE9-C73683C0D395}"/>
+  <xr:revisionPtr revIDLastSave="45" documentId="11_2843014730D8E00CF9A01B6AF2558D30C2FE69D2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37266F25-F01B-4446-BF90-FBFEB6AB8499}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Condition_GBD_mapping" sheetId="1" r:id="rId1"/>
-    <sheet name="Notes" sheetId="2" r:id="rId2"/>
+    <sheet name="User_GBD_causes" sheetId="3" r:id="rId2"/>
+    <sheet name="Notes" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Condition_GBD_mapping!$A$1:$F$34</definedName>
@@ -58,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="192">
   <si>
     <t>Karlsson_2025_priority_condition</t>
   </si>
@@ -484,13 +485,163 @@
   </si>
   <si>
     <t>Relevant for US state-level decomposition. May overlap with homicide definitions</t>
+  </si>
+  <si>
+    <t>GBD_cause_used</t>
+  </si>
+  <si>
+    <t>Karlsson_priority_condition</t>
+  </si>
+  <si>
+    <t>Karlsson_group</t>
+  </si>
+  <si>
+    <t>Classification</t>
+  </si>
+  <si>
+    <t>Alcohol use disorders</t>
+  </si>
+  <si>
+    <t>US extension</t>
+  </si>
+  <si>
+    <t>Not part of Karlsson I-8/NCD-7; relevant to U.S. mortality decomposition.</t>
+  </si>
+  <si>
+    <t>Alzheimer's disease and other dementias</t>
+  </si>
+  <si>
+    <t>Not part of Karlsson I-8/NCD-7; shown as important U.S. other-cause category.</t>
+  </si>
+  <si>
+    <t>Respiratory disease / tobacco-related sensitivity</t>
+  </si>
+  <si>
+    <t>Other / sensitivity</t>
+  </si>
+  <si>
+    <t>Not explicitly in Karlsson NCD-7 tobacco list; include as U.S. extension or sensitivity under chronic respiratory disease.</t>
+  </si>
+  <si>
+    <t>NCD-7</t>
+  </si>
+  <si>
+    <t>Listed in Karlsson supplemental table under infection-related NCDs.</t>
+  </si>
+  <si>
+    <t>Chronic hepatitis B including cirrhosis</t>
+  </si>
+  <si>
+    <t>Maps to cirrhosis due to hepatitis B.</t>
+  </si>
+  <si>
+    <t>Chronic hepatitis C including cirrhosis</t>
+  </si>
+  <si>
+    <t>Maps to cirrhosis due to hepatitis C.</t>
+  </si>
+  <si>
+    <t>Chronic kidney disease due to diabetes mellitus type 1</t>
+  </si>
+  <si>
+    <t>Maps to CKD due to diabetes.</t>
+  </si>
+  <si>
+    <t>Chronic kidney disease due to diabetes mellitus type 2</t>
+  </si>
+  <si>
+    <t>Listed in Karlsson supplemental table under tobacco-related NCDs.</t>
+  </si>
+  <si>
+    <t>Listed in Karlsson supplemental table.</t>
+  </si>
+  <si>
+    <t>Infectious 8</t>
+  </si>
+  <si>
+    <t>Childhood-cluster diseases</t>
+  </si>
+  <si>
+    <t>Part of childhood-cluster diseases.</t>
+  </si>
+  <si>
+    <t>Not part of Karlsson I-8/NCD-7; relevant U.S. extension.</t>
+  </si>
+  <si>
+    <t>HIV/AIDS and sexually transmitted infections</t>
+  </si>
+  <si>
+    <t>Use HIV/AIDS component; broader STI aggregate may need subcause filtering.</t>
+  </si>
+  <si>
+    <t>Violence</t>
+  </si>
+  <si>
+    <t>Not part of Karlsson I-8/NCD-7; shown as U.S. other-cause category.</t>
+  </si>
+  <si>
+    <t>Intracerebral hemorrhage</t>
+  </si>
+  <si>
+    <t>Haemorrhagic stroke</t>
+  </si>
+  <si>
+    <t>GBD term corresponding to hemorrhagic stroke.</t>
+  </si>
+  <si>
+    <t>Atherosclerotic CVDs</t>
+  </si>
+  <si>
+    <t>Ischemic stroke</t>
+  </si>
+  <si>
+    <t>Listed in Karlsson supplemental table under atherosclerotic CVDs.</t>
+  </si>
+  <si>
+    <t>Lip and oral cavity cancer</t>
+  </si>
+  <si>
+    <t>Maps to mouth and oropharynx cancer.</t>
+  </si>
+  <si>
+    <t>Liver cancer due to hepatitis B</t>
+  </si>
+  <si>
+    <t>Liver cancer due to hepatitis C</t>
+  </si>
+  <si>
+    <t>Mental disorders</t>
+  </si>
+  <si>
+    <t>Neurological disorders</t>
+  </si>
+  <si>
+    <t>Road injury</t>
+  </si>
+  <si>
+    <t>Suicide</t>
+  </si>
+  <si>
+    <t>Stroke aggregate</t>
+  </si>
+  <si>
+    <t>NCD-7 / aggregate</t>
+  </si>
+  <si>
+    <t>Use carefully to avoid double-counting with ischemic stroke and intracerebral hemorrhage.</t>
+  </si>
+  <si>
+    <t>Substance use disorders</t>
+  </si>
+  <si>
+    <t>Tracheal, bronchus, and lung cancer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -535,6 +686,11 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="8">
@@ -613,10 +769,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -660,11 +817,23 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{7BDFCCC1-F5B7-47B0-9E11-05EE66023C95}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -675,6 +844,20 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F08043B7-19F0-41A9-939B-5A4B319148D6}" name="UserGBDCausesTable" displayName="UserGBDCausesTable" ref="A1:E39">
+  <autoFilter ref="A1:E39" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{566E803B-F918-455F-85DB-E8404FFC6B3F}" name="GBD_cause_used"/>
+    <tableColumn id="5" xr3:uid="{EF57D0FC-5E8F-471C-81AA-F79517BF032D}" name="Classification" dataDxfId="0" dataCellStyle="Normal 2"/>
+    <tableColumn id="3" xr3:uid="{4B49F9C8-DB1C-47E6-BB7B-F6F025C6CFAA}" name="Karlsson_priority_condition"/>
+    <tableColumn id="4" xr3:uid="{3C00918F-C7B4-445B-A787-3D41E3676642}" name="Karlsson_group"/>
+    <tableColumn id="6" xr3:uid="{504517C9-0D8A-401C-B84B-AEABE6AD5675}" name="Notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1702,6 +1885,691 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A3E810A-D7CF-44E5-B5AE-F0C7DED78348}">
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="38" style="16" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" style="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29" style="16" customWidth="1"/>
+    <col min="4" max="4" width="24" style="16" customWidth="1"/>
+    <col min="5" max="5" width="55.88671875" customWidth="1"/>
+    <col min="6" max="6" width="62" style="16" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
+        <v>160</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="17" t="s">
+        <v>125</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E32" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="17" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D33" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E33" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="17" t="s">
+        <v>128</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="D34" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>131</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>